<commit_message>
Thêm âm Hán Việt cho từ vựng, hiện ở mặt sau flashcard
- Vocabulary.han_viet (VIẾT HOA, để trống = không hiện) + migration 0004
- Thẻ SC04: dòng âm Hán Việt dưới cách đọc, chỉ lộ sau khi lật; ô rỗng ẩn hẳn
- Bộ thẻ JS (study_deck) mang theo han_viet để thẻ kế tiếp cũng hiện đúng
- Admin: thêm cột + tìm kiếm; file mẫu nhập liệu và upload_vocab nhận cột mới

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/htmlTemplate/mau_danh_sach_tu_vung.xlsx
+++ b/htmlTemplate/mau_danh_sach_tu_vung.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tu_vung" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huong_dan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="tu_vung" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Huong_dan" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,13 +418,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
@@ -452,40 +452,45 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>han_viet</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>audio_url</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>topics</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>example1_jp</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>example1_vi</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>example2_jp</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>example2_vi</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>example3_jp</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>example3_vi</t>
         </is>
@@ -507,34 +512,36 @@
           <t>buổi họp, trao đổi công việc</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ĐẢ HỢP</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>hop-hanh;ho-ren-so</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>明日の打ち合わせは10時からです。</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Buổi họp ngày mai bắt đầu từ 10 giờ.</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>打ち合わせの資料を準備します。</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Tôi sẽ chuẩn bị tài liệu cho buổi họp.</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -552,26 +559,26 @@
           <t>báo giá, dự trù</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>KIẾN TÍCH</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>ban-hang-dam-phan;dat-hang-giao-nhan</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>見積もりをお願いできますか。</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Anh/chị cho tôi xin báo giá được không?</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -589,26 +596,26 @@
           <t>tôi hiểu rồi (lịch sự, dùng khi trả lời cấp trên/khách hàng)</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>THỪA TRI</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>kinh-ngu;dien-thoai</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>承知しました。すぐに対応いたします。</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Tôi hiểu rồi. Tôi sẽ xử lý ngay.</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -626,26 +633,26 @@
           <t>giao hàng, nộp hàng</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>NẠP PHẨM</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>dat-hang-giao-nhan</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>納品は来週の月曜日です。</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Việc giao hàng là vào thứ Hai tuần sau.</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -663,26 +670,26 @@
           <t>hoá đơn, giấy đề nghị thanh toán</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>THỈNH CẦU THƯ</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
         <is>
           <t>ke-toan-tai-chinh</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>請求書を送付いたします。</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Tôi xin gửi hoá đơn.</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -700,26 +707,26 @@
           <t>báo cáo</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>BÁO CÁO</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
         <is>
           <t>ho-ren-so</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>進捗を報告します。</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>Tôi xin báo cáo tiến độ.</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -737,26 +744,26 @@
           <t>tôi vô cùng xin lỗi (mức lịch sự cao nhất)</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>THÂN DỊCH</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>xin-loi-khieu-nai;kinh-ngu</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>ご迷惑をおかけし、申し訳ございません。</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>Thành thật xin lỗi vì đã làm phiền quý vị.</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -774,26 +781,26 @@
           <t>đi công tác</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>XUẤT TRƯƠNG</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>cong-tac-di-lai</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>来月大阪へ出張します。</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>Tháng sau tôi đi công tác Osaka.</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -806,7 +813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -885,193 +892,192 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>audio_url</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
+          <t>han_viet</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CharField · tối đa 200 · được để trống</t>
+          <t>CharField · tối đa 100 · được để trống · Âm Hán Việt VIẾT HOA của phần chữ Hán, vd 'CHÚ VĂN'. Để trống khi từ không có chữ Hán hoặc có chữ không có âm Hán Việt.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>topics</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
+          <t>audio_url</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Danh sách slug chủ đề, ngăn nhau bằng dấu ; — vd 'hop-hanh;dien-thoai'. Chủ đề phải có sẵn (nhập bảng vocabulary.topic trước). Chỉ THÊM liên kết còn thiếu, không gỡ liên kết đang có.</t>
+          <t>CharField · tối đa 200 · được để trống</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>example1_jp</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
+          <t>topics</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Câu ví dụ tiếng Nhật thứ 1. Điền thì phải điền cả example1_vi.</t>
+          <t>Danh sách slug chủ đề, ngăn nhau bằng dấu ; — vd 'hop-hanh;dien-thoai'. Chủ đề phải có sẵn (nhập bảng vocabulary.topic trước). Chỉ THÊM liên kết còn thiếu, không gỡ liên kết đang có.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>example1_vi</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
+          <t>example1_jp</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Nghĩa tiếng Việt của câu ví dụ thứ 1.</t>
+          <t>Câu ví dụ tiếng Nhật thứ 1. Điền thì phải điền cả example1_vi.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>example2_jp</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
+          <t>example1_vi</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Câu ví dụ tiếng Nhật thứ 2. Điền thì phải điền cả example2_vi.</t>
+          <t>Nghĩa tiếng Việt của câu ví dụ thứ 1.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>example2_vi</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
+          <t>example2_jp</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Nghĩa tiếng Việt của câu ví dụ thứ 2.</t>
+          <t>Câu ví dụ tiếng Nhật thứ 2. Điền thì phải điền cả example2_vi.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>example3_jp</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
+          <t>example2_vi</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Câu ví dụ tiếng Nhật thứ 3. Điền thì phải điền cả example3_vi.</t>
+          <t>Nghĩa tiếng Việt của câu ví dụ thứ 2.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>example3_jp</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Câu ví dụ tiếng Nhật thứ 3. Điền thì phải điền cả example3_vi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>example3_vi</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Nghĩa tiếng Việt của câu ví dụ thứ 3.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Chế độ ghi</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Chọn ngay trên màn nhập, không nằm trong file này.</t>
-        </is>
-      </c>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Chỉ thêm mới</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
+          <t>Chế độ ghi</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Dòng đã có trong hệ thống bị bỏ qua, dữ liệu cũ giữ nguyên.</t>
+          <t>Chọn ngay trên màn nhập, không nằm trong file này.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Thêm + cập nhật</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
+          <t>Chỉ thêm mới</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Dòng đã có được ghi đè theo giá trị trong file.</t>
+          <t>Dòng đã có trong hệ thống bị bỏ qua, dữ liệu cũ giữ nguyên.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Thêm + cập nhật</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Dòng đã có được ghi đè theo giá trị trong file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>Chỉ cập nhật</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Chỉ cần các cột KHOÁ; cột nào không có trong file thì field đó giữ nguyên. Cột CÓ trong file mà ô để trống = ghi giá trị rỗng/mặc định.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Khoá chống trùng</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>word, reading</t>
-        </is>
-      </c>
-    </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ghi vào 3 bảng</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
+          <t>Khoá chống trùng</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>vocabulary.vocabulary + vocabulary.vocabularytopic + vocabulary.examplesentence, tất cả trong một transaction.</t>
+          <t>word, reading</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>Ghi vào 3 bảng</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>vocabulary.vocabulary + vocabulary.vocabularytopic + vocabulary.examplesentence, tất cả trong một transaction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>Chủ đề &amp; câu ví dụ</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>CHỈ THÊM, không gỡ. Muốn bỏ bớt thì xoá ở trang quản trị Django.</t>
         </is>

</xml_diff>

<commit_message>
Từ vựng: thêm loại từ (part_of_speech), hiện ở góc phải thẻ flashcard
- Vocabulary.part_of_speech, choices lấy từ MasterCode 24 (n, n-suru, v,
  adj-i, adj-na, adv, conj, phrase, expr, other) + migration 0006
- Flashcard: nhãn loại từ ở góc phải trên thẻ (cả bộ thẻ JS), trống thì ẩn
- Admin: cột + bộ lọc loại từ; file mẫu import thêm cột part_of_speech
- upload_han_viet.py: thêm --column part_of_speech, kiểm mã theo MasterCode
- Claude outputs/loai_tu_soat.xlsx: bảng phân loại 3.036 từ đã ghi lên Supabase

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/htmlTemplate/mau_danh_sach_tu_vung.xlsx
+++ b/htmlTemplate/mau_danh_sach_tu_vung.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -455,42 +455,47 @@
           <t>han_viet</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>part_of_speech</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>audio_url</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>topics</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>example1_jp</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>example1_vi</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>example2_jp</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>example2_vi</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>example3_jp</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>example3_vi</t>
         </is>
@@ -517,27 +522,32 @@
           <t>ĐẢ HỢP</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>n-suru</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>hop-hanh;ho-ren-so</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>明日の打ち合わせは10時からです。</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Buổi họp ngày mai bắt đầu từ 10 giờ.</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>打ち合わせの資料を準備します。</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Tôi sẽ chuẩn bị tài liệu cho buổi họp.</t>
         </is>
@@ -564,17 +574,22 @@
           <t>KIẾN TÍCH</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>ban-hang-dam-phan;dat-hang-giao-nhan</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>見積もりをお願いできますか。</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Anh/chị cho tôi xin báo giá được không?</t>
         </is>
@@ -601,17 +616,22 @@
           <t>THỪA TRI</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>expr</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>kinh-ngu;dien-thoai</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>承知しました。すぐに対応いたします。</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Tôi hiểu rồi. Tôi sẽ xử lý ngay.</t>
         </is>
@@ -638,17 +658,22 @@
           <t>NẠP PHẨM</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>n-suru</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>dat-hang-giao-nhan</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>納品は来週の月曜日です。</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Việc giao hàng là vào thứ Hai tuần sau.</t>
         </is>
@@ -675,17 +700,22 @@
           <t>THỈNH CẦU THƯ</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>ke-toan-tai-chinh</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>請求書を送付いたします。</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>Tôi xin gửi hoá đơn.</t>
         </is>
@@ -712,17 +742,22 @@
           <t>BÁO CÁO</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>n-suru</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>ho-ren-so</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>進捗を報告します。</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>Tôi xin báo cáo tiến độ.</t>
         </is>
@@ -749,17 +784,22 @@
           <t>THÂN DỊCH</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>expr</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
         <is>
           <t>xin-loi-khieu-nai;kinh-ngu</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>ご迷惑をおかけし、申し訳ございません。</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>Thành thật xin lỗi vì đã làm phiền quý vị.</t>
         </is>
@@ -786,17 +826,22 @@
           <t>XUẤT TRƯƠNG</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>n-suru</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>cong-tac-di-lai</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>来月大阪へ出張します。</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>Tháng sau tôi đi công tác Osaka.</t>
         </is>
@@ -813,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -904,180 +949,192 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>audio_url</t>
+          <t>part_of_speech</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CharField · tối đa 200 · được để trống</t>
+          <t>CharField · tối đa 10 · giá trị nằm trong MasterCode · được để trống · Loại từ (MasterCode 24), vd 'adj-na'. Mã hiện ở góc phải thẻ flashcard.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>topics</t>
+          <t>audio_url</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Danh sách slug chủ đề, ngăn nhau bằng dấu ; — vd 'hop-hanh;dien-thoai'. Chủ đề phải có sẵn (nhập bảng vocabulary.topic trước). Chỉ THÊM liên kết còn thiếu, không gỡ liên kết đang có.</t>
+          <t>CharField · tối đa 200 · được để trống</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>example1_jp</t>
+          <t>topics</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Câu ví dụ tiếng Nhật thứ 1. Điền thì phải điền cả example1_vi.</t>
+          <t>Danh sách slug chủ đề, ngăn nhau bằng dấu ; — vd 'hop-hanh;dien-thoai'. Chủ đề phải có sẵn (nhập bảng vocabulary.topic trước). Chỉ THÊM liên kết còn thiếu, không gỡ liên kết đang có.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>example1_vi</t>
+          <t>example1_jp</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Nghĩa tiếng Việt của câu ví dụ thứ 1.</t>
+          <t>Câu ví dụ tiếng Nhật thứ 1. Điền thì phải điền cả example1_vi.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>example2_jp</t>
+          <t>example1_vi</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Câu ví dụ tiếng Nhật thứ 2. Điền thì phải điền cả example2_vi.</t>
+          <t>Nghĩa tiếng Việt của câu ví dụ thứ 1.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>example2_vi</t>
+          <t>example2_jp</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Nghĩa tiếng Việt của câu ví dụ thứ 2.</t>
+          <t>Câu ví dụ tiếng Nhật thứ 2. Điền thì phải điền cả example2_vi.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>example3_jp</t>
+          <t>example2_vi</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Câu ví dụ tiếng Nhật thứ 3. Điền thì phải điền cả example3_vi.</t>
+          <t>Nghĩa tiếng Việt của câu ví dụ thứ 2.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>example3_jp</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Câu ví dụ tiếng Nhật thứ 3. Điền thì phải điền cả example3_vi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>example3_vi</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Nghĩa tiếng Việt của câu ví dụ thứ 3.</t>
         </is>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Chế độ ghi</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Chọn ngay trên màn nhập, không nằm trong file này.</t>
-        </is>
-      </c>
-    </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Chỉ thêm mới</t>
+          <t>Chế độ ghi</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Dòng đã có trong hệ thống bị bỏ qua, dữ liệu cũ giữ nguyên.</t>
+          <t>Chọn ngay trên màn nhập, không nằm trong file này.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Thêm + cập nhật</t>
+          <t>Chỉ thêm mới</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Dòng đã có được ghi đè theo giá trị trong file.</t>
+          <t>Dòng đã có trong hệ thống bị bỏ qua, dữ liệu cũ giữ nguyên.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>Thêm + cập nhật</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Dòng đã có được ghi đè theo giá trị trong file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>Chỉ cập nhật</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Chỉ cần các cột KHOÁ; cột nào không có trong file thì field đó giữ nguyên. Cột CÓ trong file mà ô để trống = ghi giá trị rỗng/mặc định.</t>
         </is>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Khoá chống trùng</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>word, reading</t>
-        </is>
-      </c>
-    </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ghi vào 3 bảng</t>
+          <t>Khoá chống trùng</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>vocabulary.vocabulary + vocabulary.vocabularytopic + vocabulary.examplesentence, tất cả trong một transaction.</t>
+          <t>word, reading</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>Ghi vào 3 bảng</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>vocabulary.vocabulary + vocabulary.vocabularytopic + vocabulary.examplesentence, tất cả trong một transaction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>Chủ đề &amp; câu ví dụ</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>CHỈ THÊM, không gỡ. Muốn bỏ bớt thì xoá ở trang quản trị Django.</t>
         </is>

</xml_diff>

<commit_message>
Từ đồng nghĩa T1 + T2: model hai chiều, admin, chip trên thẻ flashcard
- VocabularySynonym (bảng nối tự trỏ, symmetrical) + Vocabulary.synonyms_note
  cho từ ngoài hệ thống; save()/delete() tự giữ dòng chiều ngược; migration 0008.
- Admin: inline đồng nghĩa (autocomplete); dataio khoá (vocabulary, synonym);
  cột synonyms_note thêm vào file mẫu mau_danh_sach_tu_vung.{csv,xlsx}.
- _card_extra.html: chip đồng nghĩa dưới thẻ (tối đa 5, từ trong hệ thống mở
  SC05 ở tab mới), "Chưa có ví dụ cho từ này" khi không có ví dụ (◆4).
- get_study_cards prefetch synonyms; test số query không tăng theo số thẻ.
- Sửa test dataio cũ chưa tính cột ExampleSentence.audio_url.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/htmlTemplate/mau_danh_sach_tu_vung.xlsx
+++ b/htmlTemplate/mau_danh_sach_tu_vung.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -465,37 +465,42 @@
           <t>audio_url</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>synonyms_note</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>topics</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>example1_jp</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>example1_vi</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>example2_jp</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>example2_vi</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>example3_jp</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>example3_vi</t>
         </is>
@@ -527,27 +532,27 @@
           <t>n-suru</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>hop-hanh;ho-ren-so</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>明日の打ち合わせは10時からです。</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Buổi họp ngày mai bắt đầu từ 10 giờ.</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>打ち合わせの資料を準備します。</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Tôi sẽ chuẩn bị tài liệu cho buổi họp.</t>
         </is>
@@ -579,17 +584,17 @@
           <t>n</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>ban-hang-dam-phan;dat-hang-giao-nhan</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>見積もりをお願いできますか。</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Anh/chị cho tôi xin báo giá được không?</t>
         </is>
@@ -621,17 +626,17 @@
           <t>expr</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>kinh-ngu;dien-thoai</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>承知しました。すぐに対応いたします。</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Tôi hiểu rồi. Tôi sẽ xử lý ngay.</t>
         </is>
@@ -663,17 +668,17 @@
           <t>n-suru</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>dat-hang-giao-nhan</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>納品は来週の月曜日です。</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Việc giao hàng là vào thứ Hai tuần sau.</t>
         </is>
@@ -705,17 +710,17 @@
           <t>n</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>ke-toan-tai-chinh</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>請求書を送付いたします。</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Tôi xin gửi hoá đơn.</t>
         </is>
@@ -747,17 +752,17 @@
           <t>n-suru</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>ho-ren-so</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>進捗を報告します。</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Tôi xin báo cáo tiến độ.</t>
         </is>
@@ -789,17 +794,17 @@
           <t>expr</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>xin-loi-khieu-nai;kinh-ngu</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>ご迷惑をおかけし、申し訳ございません。</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Thành thật xin lỗi vì đã làm phiền quý vị.</t>
         </is>
@@ -831,17 +836,17 @@
           <t>n-suru</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>cong-tac-di-lai</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>来月大阪へ出張します。</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Tháng sau tôi đi công tác Osaka.</t>
         </is>
@@ -1054,7 +1059,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -1103,7 +1107,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>

</xml_diff>